<commit_message>
fix(schedule): заменить Calibri на Times New Roman в файлах xlsx
Тема, которую ClosedXML и шаблоны Excel подставляют по умолчанию, — Calibri,
поэтому в выгрузках и в раздаваемых шаблонах документы выглядели неоднородно.

Статические файлы: Calibri вычищен из таблицы шрифтов styles.xml и из темы
theme1.xml (major и minor), у шрифтов с scheme="minor" scheme убран, family
2→1 — иначе Excel возвращает шрифт по умолчанию из темы. Матрица расписания,
объединённые ячейки и закрепление столбцов не изменились.

Выгрузки: стиль книги не переживает сериализацию, поэтому шрифт задаётся
явно на всю заполненную область листа через XlsxDefaults.ApplyFont.
Исторические файлы в import/schedule/Корректировки не тронуты: это fixtures
тестов и записи того, что прислал колледж.
</commit_message>
<xml_diff>
--- a/import/schedule/Корректировка.xlsx
+++ b/import/schedule/Корректировка.xlsx
@@ -121,9 +121,8 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
@@ -514,7 +513,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Times New Roman" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="Yu Gothic Light"/>
@@ -549,7 +548,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Times New Roman" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="Yu Gothic"/>

</xml_diff>